<commit_message>
feat(tms): update template files
</commit_message>
<xml_diff>
--- a/first-mile/src/main/resources/excel/order_template.xlsx
+++ b/first-mile/src/main/resources/excel/order_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\hanh chinh vn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BDF612-E033-47C7-B7A8-E283163182B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01D5725-2BF0-4EF2-81D5-CA3010C9A2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCEF8B10-CC32-4706-81E7-C863D6A361A9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3422" uniqueCount="3407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3445" uniqueCount="3423">
   <si>
     <t>Phường/xã</t>
   </si>
@@ -10258,6 +10258,54 @@
   </si>
   <si>
     <t>DOCHOI - Đồ chơi</t>
+  </si>
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>ANHNTA-01</t>
+  </si>
+  <si>
+    <t>0966277109</t>
+  </si>
+  <si>
+    <t>Thôn Miếu</t>
+  </si>
+  <si>
+    <t>Nguyễn Thế Anh</t>
+  </si>
+  <si>
+    <t>ĐHBKHN</t>
+  </si>
+  <si>
+    <t>0979264109</t>
+  </si>
+  <si>
+    <t>Đại học Bách khoa Hà Nội</t>
+  </si>
+  <si>
+    <t>test note</t>
+  </si>
+  <si>
+    <t>01/04/2026</t>
+  </si>
+  <si>
+    <t>5 x 6 x 7</t>
+  </si>
+  <si>
+    <t>Bim bim</t>
+  </si>
+  <si>
+    <t>20000</t>
+  </si>
+  <si>
+    <t>30000</t>
+  </si>
+  <si>
+    <t>Sữa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -10346,7 +10394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -10366,6 +10414,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10700,54 +10750,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EB74871-DFC8-4C09-A84E-833370EABA59}">
-  <dimension ref="A2:AD4"/>
+  <dimension ref="A2:AE5"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="17.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5546875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.77734375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="21.88671875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="14.109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="25.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="32.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.6640625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="22.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.77734375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="25.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="32.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.6640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:30" s="3" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="1:31" s="3" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="8"/>
+      <c r="H2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="8"/>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="8"/>
       <c r="N2" s="8"/>
       <c r="O2" s="8"/>
       <c r="P2" s="8"/>
@@ -10756,176 +10808,272 @@
       <c r="S2" s="8"/>
       <c r="T2" s="8"/>
       <c r="U2" s="8"/>
-      <c r="V2" s="8" t="s">
+      <c r="V2" s="8"/>
+      <c r="W2" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="W2" s="8"/>
       <c r="X2" s="8"/>
       <c r="Y2" s="8"/>
       <c r="Z2" s="8"/>
-      <c r="AA2" s="1"/>
+      <c r="AA2" s="8"/>
       <c r="AB2" s="1"/>
-      <c r="AC2" s="7"/>
-    </row>
-    <row r="3" spans="1:30" s="5" customFormat="1" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="7"/>
+    </row>
+    <row r="3" spans="1:31" s="5" customFormat="1" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>3407</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="L3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="N3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="O3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="U3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="V3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="X3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="X3" s="4" t="s">
+      <c r="Y3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" s="4" t="s">
+      <c r="Z3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Z3" s="4" t="s">
+      <c r="AA3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="D4" s="1" t="s">
-        <v>3372</v>
-      </c>
-      <c r="P4" s="1" t="s">
+      <c r="AE3" s="6"/>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3408</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3411</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>3409</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>3376</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>2857</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>3410</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3412</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>3413</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>3392</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>3414</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>3415</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>3416</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="U4" s="1" t="s">
+      <c r="T4" s="1" t="s">
+        <v>3417</v>
+      </c>
+      <c r="U4" s="1">
+        <v>1</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>3418</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>3419</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>2</v>
+      </c>
+      <c r="Z4" s="1">
+        <v>20</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>3406</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>3422</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>3421</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>3420</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>3</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>30</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>3404</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="L2:U2"/>
-    <mergeCell ref="V2:Z2"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="M2:V2"/>
+    <mergeCell ref="W2:AA2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FE4D717C-EE07-4F4E-8D19-0FCBDC9810E8}">
           <x14:formula1>
             <xm:f>Unit!$B$2:$B$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>D4:D1048576 I4:I1048576</xm:sqref>
+          <xm:sqref>E4:E1048576 J4:J1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{78016778-AB15-4BDA-B8B5-5AFA12D85284}">
           <x14:formula1>
             <xm:f>Unit!$A$2:$A$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>E4:E1048576 J4:J1048576</xm:sqref>
+          <xm:sqref>F4:F1048576 K4:K1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D69BF08A-0999-4E54-AD15-003C8B3C4E86}">
           <x14:formula1>
             <xm:f>Unit!$C$2:$C$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>L4:L1048576</xm:sqref>
+          <xm:sqref>M4:M1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{13F3EB98-3A35-48E6-A4CB-9C7C7D50576B}">
           <x14:formula1>
             <xm:f>Unit!$D$2:$D$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>M6:M1048576 M4</xm:sqref>
+          <xm:sqref>N6:N1048576 N4</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A5B2618A-5CA9-4FC0-B534-1DB7CABF11BA}">
           <x14:formula1>
             <xm:f>Unit!$H$2:$H$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>P4:P1048576</xm:sqref>
+          <xm:sqref>Q4:Q1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2014D110-843A-4F16-A6AE-EC962F4F7DD3}">
           <x14:formula1>
             <xm:f>Unit!$I$2:$I$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>Q4:Q1048576</xm:sqref>
+          <xm:sqref>R4:R1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6B7A4CDC-3098-4E66-A942-2A6A27C6E072}">
           <x14:formula1>
             <xm:f>Unit!$G$2:$G$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>R4:R1048576</xm:sqref>
+          <xm:sqref>S4:S1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0269EBB6-0703-4D5E-9141-69EBCE5241FC}">
           <x14:formula1>
             <xm:f>Unit!$E$2:$E$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>U4:U1048576</xm:sqref>
+          <xm:sqref>V4:V1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FC2DA025-C28A-43BB-98DC-B77683BAF21D}">
+          <x14:formula1>
+            <xm:f>Unit!$F$2:$F$1000000</xm:f>
+          </x14:formula1>
+          <xm:sqref>AA4:AA1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>